<commit_message>
ajout MI mobilité publique
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projects/critical_materials/excel_files/Recycling_rates.xlsx
+++ b/projects/critical_materials/excel_files/Recycling_rates.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Paolo/Documents/PdM_code/EnergyScope-Quebec/projects/critical_materials/excel_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98923B30-9BE2-CE45-9A2F-EC293B7ECE40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5062E829-1B26-0847-81C6-A8D9828FFB66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="37960" windowHeight="19500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="37960" windowHeight="19500" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table of content" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <sheet name="RR_Vehicles_Public" sheetId="8" r:id="rId5"/>
     <sheet name="RR_H2" sheetId="9" r:id="rId6"/>
     <sheet name="Recycling_scenario" sheetId="16" r:id="rId7"/>
-    <sheet name="Recycling_scenario_technologies" sheetId="22" r:id="rId8"/>
+    <sheet name="Collection_rate" sheetId="22" r:id="rId8"/>
     <sheet name="Recycling_technologies" sheetId="17" r:id="rId9"/>
     <sheet name="Recycling_cost" sheetId="20" r:id="rId10"/>
     <sheet name="Electricity_use" sheetId="21" r:id="rId11"/>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3413" uniqueCount="1061">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3433" uniqueCount="1061">
   <si>
     <t>Sol_C-si_Silver</t>
   </si>
@@ -4125,7 +4125,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="160">
+  <cellXfs count="158">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -4303,7 +4303,6 @@
     <xf numFmtId="10" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="10" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="2"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="2" fillId="8" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4332,6 +4331,10 @@
     <xf numFmtId="10" fontId="17" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="8" fillId="38" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="10" fontId="0" fillId="33" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -4391,11 +4394,6 @@
     <xf numFmtId="0" fontId="0" fillId="30" borderId="26" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="34" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="33" borderId="7" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Lien hypertexte" xfId="2" builtinId="8"/>
@@ -4693,18 +4691,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="14.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="135" t="s">
+      <c r="A1" s="138" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="136"/>
+      <c r="B1" s="139"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A2" s="137"/>
-      <c r="B2" s="138"/>
+      <c r="A2" s="140"/>
+      <c r="B2" s="141"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="139"/>
-      <c r="B3" s="140"/>
+      <c r="A3" s="142"/>
+      <c r="B3" s="143"/>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="11" t="s">
@@ -4713,10 +4711,10 @@
       <c r="B4" s="30"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="146" t="s">
+      <c r="A5" s="149" t="s">
         <v>32</v>
       </c>
-      <c r="B5" s="131"/>
+      <c r="B5" s="134"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" s="12" t="s">
@@ -4727,10 +4725,10 @@
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="143" t="s">
+      <c r="A7" s="146" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="131"/>
+      <c r="B7" s="134"/>
     </row>
     <row r="8" spans="1:2" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="25" t="s">
@@ -4757,13 +4755,13 @@
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A11" s="145" t="s">
+      <c r="A11" s="148" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="131"/>
+      <c r="B11" s="134"/>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="142" t="s">
+      <c r="A12" s="145" t="s">
         <v>43</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -4771,13 +4769,13 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="133"/>
+      <c r="A13" s="136"/>
       <c r="B13" s="3" t="s">
         <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="134"/>
+      <c r="A14" s="137"/>
       <c r="B14" s="3" t="s">
         <v>46</v>
       </c>
@@ -4815,10 +4813,10 @@
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A19" s="144" t="s">
+      <c r="A19" s="147" t="s">
         <v>55</v>
       </c>
-      <c r="B19" s="131"/>
+      <c r="B19" s="134"/>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" s="24" t="s">
@@ -4829,7 +4827,7 @@
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A21" s="141" t="s">
+      <c r="A21" s="144" t="s">
         <v>58</v>
       </c>
       <c r="B21" s="3" t="s">
@@ -4837,19 +4835,19 @@
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A22" s="134"/>
+      <c r="A22" s="137"/>
       <c r="B22" s="3" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A23" s="132" t="s">
+      <c r="A23" s="135" t="s">
         <v>61</v>
       </c>
-      <c r="B23" s="131"/>
+      <c r="B23" s="134"/>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A24" s="132" t="s">
+      <c r="A24" s="135" t="s">
         <v>62</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -4857,19 +4855,19 @@
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A25" s="133"/>
+      <c r="A25" s="136"/>
       <c r="B25" s="3" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A26" s="133"/>
+      <c r="A26" s="136"/>
       <c r="B26" s="3" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A27" s="134"/>
+      <c r="A27" s="137"/>
       <c r="B27" s="3" t="s">
         <v>66</v>
       </c>
@@ -4907,10 +4905,10 @@
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A32" s="130" t="s">
+      <c r="A32" s="133" t="s">
         <v>75</v>
       </c>
-      <c r="B32" s="131"/>
+      <c r="B32" s="134"/>
     </row>
     <row r="33" spans="1:2" ht="32" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="19" t="s">
@@ -4967,7 +4965,7 @@
       <c r="C1" s="21" t="s">
         <v>919</v>
       </c>
-      <c r="D1" s="110" t="s">
+      <c r="D1" s="109" t="s">
         <v>1016</v>
       </c>
       <c r="E1" s="31" t="s">
@@ -5002,28 +5000,28 @@
       <c r="C2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D2" s="111" t="s">
+      <c r="D2" s="110" t="s">
         <v>1017</v>
       </c>
-      <c r="E2" s="125">
+      <c r="E2" s="124">
         <v>95.24</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>1008</v>
       </c>
-      <c r="G2" s="125">
+      <c r="G2" s="124">
         <v>0.90500000000000003</v>
       </c>
       <c r="H2" s="4" t="s">
         <v>1025</v>
       </c>
-      <c r="I2" s="113" t="s">
+      <c r="I2" s="112" t="s">
         <v>1027</v>
       </c>
-      <c r="J2" s="114" t="s">
+      <c r="J2" s="113" t="s">
         <v>1026</v>
       </c>
-      <c r="K2" s="113" t="s">
+      <c r="K2" s="112" t="s">
         <v>1054</v>
       </c>
     </row>
@@ -5037,28 +5035,28 @@
       <c r="C3" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D3" s="111" t="s">
+      <c r="D3" s="110" t="s">
         <v>1022</v>
       </c>
-      <c r="E3" s="125">
+      <c r="E3" s="124">
         <v>123.06</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>1008</v>
       </c>
-      <c r="G3" s="125">
+      <c r="G3" s="124">
         <v>1.3393999999999999</v>
       </c>
       <c r="H3" s="4" t="s">
         <v>1025</v>
       </c>
-      <c r="I3" s="113" t="s">
+      <c r="I3" s="112" t="s">
         <v>1027</v>
       </c>
-      <c r="J3" s="114" t="s">
+      <c r="J3" s="113" t="s">
         <v>1026</v>
       </c>
-      <c r="K3" s="113" t="s">
+      <c r="K3" s="112" t="s">
         <v>1042</v>
       </c>
     </row>
@@ -5072,46 +5070,46 @@
       <c r="C4" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D4" s="111" t="s">
+      <c r="D4" s="110" t="s">
         <v>1044</v>
       </c>
-      <c r="E4" s="125">
+      <c r="E4" s="124">
         <v>150</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>1008</v>
       </c>
-      <c r="G4" s="125">
+      <c r="G4" s="124">
         <v>1.64</v>
       </c>
       <c r="H4" s="4" t="s">
         <v>1025</v>
       </c>
-      <c r="I4" s="113"/>
-      <c r="J4" s="114"/>
-      <c r="K4" s="113" t="s">
+      <c r="I4" s="112"/>
+      <c r="J4" s="113"/>
+      <c r="K4" s="112" t="s">
         <v>1053</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D5"/>
-      <c r="J5" s="115"/>
+      <c r="J5" s="114"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D6"/>
-      <c r="J6" s="115"/>
+      <c r="J6" s="114"/>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D7"/>
-      <c r="J7" s="115"/>
+      <c r="J7" s="114"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D8"/>
-      <c r="J8" s="115"/>
+      <c r="J8" s="114"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D9"/>
-      <c r="J9" s="115"/>
+      <c r="J9" s="114"/>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.2">
       <c r="D10"/>
@@ -5147,7 +5145,7 @@
       <c r="C1" s="21" t="s">
         <v>919</v>
       </c>
-      <c r="D1" s="110" t="s">
+      <c r="D1" s="109" t="s">
         <v>1016</v>
       </c>
       <c r="E1" s="31" t="s">
@@ -5176,10 +5174,10 @@
       <c r="C2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D2" s="111" t="s">
+      <c r="D2" s="110" t="s">
         <v>1017</v>
       </c>
-      <c r="E2" s="105" t="s">
+      <c r="E2" s="104" t="s">
         <v>1031</v>
       </c>
       <c r="F2" s="4" t="s">
@@ -5188,7 +5186,7 @@
       <c r="G2" s="3" t="s">
         <v>1032</v>
       </c>
-      <c r="H2" s="107" t="s">
+      <c r="H2" s="106" t="s">
         <v>1033</v>
       </c>
       <c r="I2" s="3" t="s">
@@ -5236,7 +5234,7 @@
       <c r="B2">
         <v>3010</v>
       </c>
-      <c r="C2" s="104" t="s">
+      <c r="C2" s="103" t="s">
         <v>947</v>
       </c>
       <c r="D2" t="s">
@@ -16212,7 +16210,10 @@
         <v>882</v>
       </c>
       <c r="B692" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D692" t="s">
+        <v>9</v>
       </c>
       <c r="H692" s="36" t="s">
         <v>181</v>
@@ -16223,7 +16224,10 @@
         <v>883</v>
       </c>
       <c r="B693" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D693" t="s">
+        <v>10</v>
       </c>
       <c r="H693" s="36" t="s">
         <v>181</v>
@@ -16234,7 +16238,10 @@
         <v>884</v>
       </c>
       <c r="B694" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D694" t="s">
+        <v>11</v>
       </c>
       <c r="H694" s="36" t="s">
         <v>181</v>
@@ -16245,7 +16252,10 @@
         <v>885</v>
       </c>
       <c r="B695" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D695" t="s">
+        <v>12</v>
       </c>
       <c r="H695" s="36" t="s">
         <v>181</v>
@@ -16256,7 +16266,10 @@
         <v>886</v>
       </c>
       <c r="B696" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D696" t="s">
+        <v>9</v>
       </c>
       <c r="H696" s="36" t="s">
         <v>181</v>
@@ -16267,7 +16280,10 @@
         <v>887</v>
       </c>
       <c r="B697" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D697" t="s">
+        <v>10</v>
       </c>
       <c r="H697" s="36" t="s">
         <v>181</v>
@@ -16278,7 +16294,10 @@
         <v>888</v>
       </c>
       <c r="B698" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D698" t="s">
+        <v>11</v>
       </c>
       <c r="H698" s="36" t="s">
         <v>181</v>
@@ -16289,7 +16308,10 @@
         <v>889</v>
       </c>
       <c r="B699" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D699" t="s">
+        <v>12</v>
       </c>
       <c r="H699" s="36" t="s">
         <v>181</v>
@@ -16300,7 +16322,10 @@
         <v>890</v>
       </c>
       <c r="B700" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D700" t="s">
+        <v>13</v>
       </c>
       <c r="H700" s="36" t="s">
         <v>181</v>
@@ -16311,7 +16336,10 @@
         <v>891</v>
       </c>
       <c r="B701" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D701" t="s">
+        <v>14</v>
       </c>
       <c r="H701" s="36" t="s">
         <v>181</v>
@@ -16322,7 +16350,10 @@
         <v>892</v>
       </c>
       <c r="B702" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D702" t="s">
+        <v>15</v>
       </c>
       <c r="H702" s="36" t="s">
         <v>181</v>
@@ -16333,7 +16364,10 @@
         <v>893</v>
       </c>
       <c r="B703" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D703" t="s">
+        <v>16</v>
       </c>
       <c r="H703" s="36" t="s">
         <v>181</v>
@@ -16344,7 +16378,10 @@
         <v>894</v>
       </c>
       <c r="B704" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D704" t="s">
+        <v>0</v>
       </c>
       <c r="H704" s="36" t="s">
         <v>181</v>
@@ -16355,7 +16392,10 @@
         <v>895</v>
       </c>
       <c r="B705" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D705" t="s">
+        <v>2</v>
       </c>
       <c r="H705" s="36" t="s">
         <v>181</v>
@@ -16366,7 +16406,10 @@
         <v>896</v>
       </c>
       <c r="B706" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D706" t="s">
+        <v>3</v>
       </c>
       <c r="H706" s="36" t="s">
         <v>181</v>
@@ -16377,7 +16420,10 @@
         <v>897</v>
       </c>
       <c r="B707" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D707" t="s">
+        <v>4</v>
       </c>
       <c r="H707" s="36" t="s">
         <v>181</v>
@@ -16388,7 +16434,10 @@
         <v>898</v>
       </c>
       <c r="B708" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D708" t="s">
+        <v>0</v>
       </c>
       <c r="H708" s="36" t="s">
         <v>181</v>
@@ -16399,7 +16448,10 @@
         <v>899</v>
       </c>
       <c r="B709" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D709" t="s">
+        <v>2</v>
       </c>
       <c r="H709" s="36" t="s">
         <v>181</v>
@@ -16410,7 +16462,10 @@
         <v>900</v>
       </c>
       <c r="B710" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D710" t="s">
+        <v>3</v>
       </c>
       <c r="H710" s="36" t="s">
         <v>181</v>
@@ -16421,7 +16476,10 @@
         <v>901</v>
       </c>
       <c r="B711" s="35" t="s">
-        <v>180</v>
+        <v>187</v>
+      </c>
+      <c r="D711" t="s">
+        <v>4</v>
       </c>
       <c r="H711" s="36" t="s">
         <v>181</v>
@@ -16508,13 +16566,13 @@
       <c r="B1" s="21" t="s">
         <v>918</v>
       </c>
-      <c r="C1" s="110" t="s">
+      <c r="C1" s="109" t="s">
         <v>919</v>
       </c>
-      <c r="D1" s="110" t="s">
+      <c r="D1" s="109" t="s">
         <v>1016</v>
       </c>
-      <c r="E1" s="106" t="s">
+      <c r="E1" s="105" t="s">
         <v>1003</v>
       </c>
       <c r="F1" s="21" t="s">
@@ -16534,16 +16592,16 @@
       <c r="A2" s="3" t="s">
         <v>1005</v>
       </c>
-      <c r="B2" s="108" t="s">
+      <c r="B2" s="107" t="s">
         <v>1006</v>
       </c>
       <c r="C2" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="D2" s="111" t="s">
+      <c r="D2" s="110" t="s">
         <v>1017</v>
       </c>
-      <c r="E2" s="109">
+      <c r="E2" s="108">
         <v>0.95</v>
       </c>
       <c r="F2" s="4" t="s">
@@ -16552,7 +16610,7 @@
       <c r="G2" s="3" t="s">
         <v>1011</v>
       </c>
-      <c r="H2" s="107" t="s">
+      <c r="H2" s="106" t="s">
         <v>1010</v>
       </c>
       <c r="I2" s="3"/>
@@ -16561,16 +16619,16 @@
       <c r="A3" s="3" t="s">
         <v>1005</v>
       </c>
-      <c r="B3" s="108" t="s">
+      <c r="B3" s="107" t="s">
         <v>1006</v>
       </c>
       <c r="C3" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="D3" s="111" t="s">
+      <c r="D3" s="110" t="s">
         <v>1017</v>
       </c>
-      <c r="E3" s="112">
+      <c r="E3" s="111">
         <v>0.95</v>
       </c>
       <c r="F3" s="4" t="s">
@@ -16579,7 +16637,7 @@
       <c r="G3" s="3" t="s">
         <v>1012</v>
       </c>
-      <c r="H3" s="107" t="s">
+      <c r="H3" s="106" t="s">
         <v>1013</v>
       </c>
       <c r="I3" s="3"/>
@@ -16588,16 +16646,16 @@
       <c r="A4" s="3" t="s">
         <v>1005</v>
       </c>
-      <c r="B4" s="108" t="s">
+      <c r="B4" s="107" t="s">
         <v>1006</v>
       </c>
       <c r="C4" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="D4" s="111" t="s">
+      <c r="D4" s="110" t="s">
         <v>1017</v>
       </c>
-      <c r="E4" s="109">
+      <c r="E4" s="108">
         <v>0.97</v>
       </c>
       <c r="F4" s="4" t="s">
@@ -16606,7 +16664,7 @@
       <c r="G4" s="3" t="s">
         <v>1014</v>
       </c>
-      <c r="H4" s="107" t="s">
+      <c r="H4" s="106" t="s">
         <v>1015</v>
       </c>
       <c r="I4" s="3"/>
@@ -16615,16 +16673,16 @@
       <c r="A5" s="3" t="s">
         <v>1005</v>
       </c>
-      <c r="B5" s="108" t="s">
+      <c r="B5" s="107" t="s">
         <v>1006</v>
       </c>
       <c r="C5" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="D5" s="111" t="s">
+      <c r="D5" s="110" t="s">
         <v>1017</v>
       </c>
-      <c r="E5" s="112">
+      <c r="E5" s="111">
         <v>0.41</v>
       </c>
       <c r="F5" s="4" t="s">
@@ -16633,7 +16691,7 @@
       <c r="G5" s="2" t="s">
         <v>1018</v>
       </c>
-      <c r="H5" s="107" t="s">
+      <c r="H5" s="106" t="s">
         <v>1020</v>
       </c>
       <c r="I5" s="3"/>
@@ -16642,16 +16700,16 @@
       <c r="A6" s="3" t="s">
         <v>1005</v>
       </c>
-      <c r="B6" s="108" t="s">
+      <c r="B6" s="107" t="s">
         <v>1006</v>
       </c>
       <c r="C6" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D6" s="111" t="s">
+      <c r="D6" s="110" t="s">
         <v>1017</v>
       </c>
-      <c r="E6" s="109">
+      <c r="E6" s="108">
         <v>0.74</v>
       </c>
       <c r="F6" s="4" t="s">
@@ -16660,7 +16718,7 @@
       <c r="G6" s="2" t="s">
         <v>1018</v>
       </c>
-      <c r="H6" s="107" t="s">
+      <c r="H6" s="106" t="s">
         <v>1021</v>
       </c>
       <c r="I6" s="3"/>
@@ -16669,16 +16727,16 @@
       <c r="A7" s="3" t="s">
         <v>1005</v>
       </c>
-      <c r="B7" s="108" t="s">
+      <c r="B7" s="107" t="s">
         <v>1006</v>
       </c>
       <c r="C7" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="D7" s="111" t="s">
+      <c r="D7" s="110" t="s">
         <v>1017</v>
       </c>
-      <c r="E7" s="109">
+      <c r="E7" s="108">
         <v>0.92</v>
       </c>
       <c r="F7" s="4" t="s">
@@ -16687,7 +16745,7 @@
       <c r="G7" s="2" t="s">
         <v>1018</v>
       </c>
-      <c r="H7" s="107" t="s">
+      <c r="H7" s="106" t="s">
         <v>1019</v>
       </c>
       <c r="I7" s="3"/>
@@ -16696,16 +16754,16 @@
       <c r="A8" s="3" t="s">
         <v>1005</v>
       </c>
-      <c r="B8" s="108" t="s">
+      <c r="B8" s="107" t="s">
         <v>1006</v>
       </c>
       <c r="C8" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="111" t="s">
+      <c r="D8" s="110" t="s">
         <v>1022</v>
       </c>
-      <c r="E8" s="109">
+      <c r="E8" s="108">
         <v>0.99970000000000003</v>
       </c>
       <c r="F8" s="4" t="s">
@@ -16714,7 +16772,7 @@
       <c r="G8" s="2" t="s">
         <v>1035</v>
       </c>
-      <c r="H8" s="122" t="s">
+      <c r="H8" s="121" t="s">
         <v>1036</v>
       </c>
       <c r="I8" s="3"/>
@@ -16723,16 +16781,16 @@
       <c r="A9" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B9" s="118" t="s">
+      <c r="B9" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C9" s="119" t="s">
+      <c r="C9" s="118" t="s">
         <v>91</v>
       </c>
-      <c r="D9" s="120" t="s">
+      <c r="D9" s="119" t="s">
         <v>1022</v>
       </c>
-      <c r="E9" s="121">
+      <c r="E9" s="120">
         <v>1</v>
       </c>
       <c r="F9" s="93" t="s">
@@ -16741,7 +16799,7 @@
       <c r="G9" s="2" t="s">
         <v>1035</v>
       </c>
-      <c r="H9" s="122" t="s">
+      <c r="H9" s="121" t="s">
         <v>1036</v>
       </c>
       <c r="I9" s="54"/>
@@ -16750,16 +16808,16 @@
       <c r="A10" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B10" s="118" t="s">
+      <c r="B10" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C10" s="119" t="s">
+      <c r="C10" s="118" t="s">
         <v>135</v>
       </c>
-      <c r="D10" s="120" t="s">
+      <c r="D10" s="119" t="s">
         <v>1022</v>
       </c>
-      <c r="E10" s="121">
+      <c r="E10" s="120">
         <v>1</v>
       </c>
       <c r="F10" s="93" t="s">
@@ -16768,7 +16826,7 @@
       <c r="G10" s="2" t="s">
         <v>1035</v>
       </c>
-      <c r="H10" s="122" t="s">
+      <c r="H10" s="121" t="s">
         <v>1036</v>
       </c>
       <c r="I10" s="54"/>
@@ -16777,16 +16835,16 @@
       <c r="A11" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B11" s="118" t="s">
+      <c r="B11" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C11" s="119" t="s">
+      <c r="C11" s="118" t="s">
         <v>108</v>
       </c>
-      <c r="D11" s="120" t="s">
+      <c r="D11" s="119" t="s">
         <v>1022</v>
       </c>
-      <c r="E11" s="121">
+      <c r="E11" s="120">
         <v>0.98</v>
       </c>
       <c r="F11" s="93" t="s">
@@ -16795,7 +16853,7 @@
       <c r="G11" s="2" t="s">
         <v>1035</v>
       </c>
-      <c r="H11" s="122" t="s">
+      <c r="H11" s="121" t="s">
         <v>1036</v>
       </c>
       <c r="I11" s="54"/>
@@ -16804,16 +16862,16 @@
       <c r="A12" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B12" s="118" t="s">
+      <c r="B12" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C12" s="119" t="s">
+      <c r="C12" s="118" t="s">
         <v>137</v>
       </c>
-      <c r="D12" s="120" t="s">
+      <c r="D12" s="119" t="s">
         <v>1022</v>
       </c>
-      <c r="E12" s="124">
+      <c r="E12" s="123">
         <v>0.32</v>
       </c>
       <c r="F12" s="93" t="s">
@@ -16822,7 +16880,7 @@
       <c r="G12" s="2" t="s">
         <v>1035</v>
       </c>
-      <c r="H12" s="122" t="s">
+      <c r="H12" s="121" t="s">
         <v>1036</v>
       </c>
       <c r="I12" s="54"/>
@@ -16831,16 +16889,16 @@
       <c r="A13" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B13" s="118" t="s">
+      <c r="B13" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C13" s="119" t="s">
+      <c r="C13" s="118" t="s">
         <v>99</v>
       </c>
-      <c r="D13" s="120" t="s">
+      <c r="D13" s="119" t="s">
         <v>1022</v>
       </c>
-      <c r="E13" s="121">
+      <c r="E13" s="120">
         <v>0.89</v>
       </c>
       <c r="F13" s="93" t="s">
@@ -16849,7 +16907,7 @@
       <c r="G13" s="2" t="s">
         <v>1037</v>
       </c>
-      <c r="H13" s="122" t="s">
+      <c r="H13" s="121" t="s">
         <v>1039</v>
       </c>
       <c r="I13" s="54"/>
@@ -16858,16 +16916,16 @@
       <c r="A14" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B14" s="118" t="s">
+      <c r="B14" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C14" s="119" t="s">
+      <c r="C14" s="118" t="s">
         <v>80</v>
       </c>
-      <c r="D14" s="120" t="s">
+      <c r="D14" s="119" t="s">
         <v>1022</v>
       </c>
-      <c r="E14" s="121">
+      <c r="E14" s="120">
         <v>0.81</v>
       </c>
       <c r="F14" s="93" t="s">
@@ -16876,7 +16934,7 @@
       <c r="G14" s="2" t="s">
         <v>1037</v>
       </c>
-      <c r="H14" s="122" t="s">
+      <c r="H14" s="121" t="s">
         <v>1040</v>
       </c>
       <c r="I14" s="54"/>
@@ -16885,16 +16943,16 @@
       <c r="A15" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B15" s="118" t="s">
+      <c r="B15" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C15" s="119" t="s">
+      <c r="C15" s="118" t="s">
         <v>135</v>
       </c>
-      <c r="D15" s="120" t="s">
+      <c r="D15" s="119" t="s">
         <v>1022</v>
       </c>
-      <c r="E15" s="121">
+      <c r="E15" s="120">
         <v>0.8</v>
       </c>
       <c r="F15" s="93" t="s">
@@ -16903,7 +16961,7 @@
       <c r="G15" s="2" t="s">
         <v>1037</v>
       </c>
-      <c r="H15" s="122" t="s">
+      <c r="H15" s="121" t="s">
         <v>1041</v>
       </c>
       <c r="I15" s="54"/>
@@ -16912,16 +16970,16 @@
       <c r="A16" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B16" s="118" t="s">
+      <c r="B16" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C16" s="119" t="s">
+      <c r="C16" s="118" t="s">
         <v>137</v>
       </c>
-      <c r="D16" s="120" t="s">
+      <c r="D16" s="119" t="s">
         <v>1022</v>
       </c>
-      <c r="E16" s="124">
+      <c r="E16" s="123">
         <v>0.89</v>
       </c>
       <c r="F16" s="93" t="s">
@@ -16930,7 +16988,7 @@
       <c r="G16" s="2" t="s">
         <v>1037</v>
       </c>
-      <c r="H16" s="122" t="s">
+      <c r="H16" s="121" t="s">
         <v>1038</v>
       </c>
       <c r="I16" s="54"/>
@@ -16939,16 +16997,16 @@
       <c r="A17" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B17" s="118" t="s">
+      <c r="B17" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C17" s="119" t="s">
+      <c r="C17" s="118" t="s">
         <v>91</v>
       </c>
-      <c r="D17" s="120" t="s">
+      <c r="D17" s="119" t="s">
         <v>1044</v>
       </c>
-      <c r="E17" s="128">
+      <c r="E17" s="127">
         <v>0.83</v>
       </c>
       <c r="F17" s="93" t="s">
@@ -16957,7 +17015,7 @@
       <c r="G17" s="2" t="s">
         <v>1047</v>
       </c>
-      <c r="H17" s="122" t="s">
+      <c r="H17" s="121" t="s">
         <v>1046</v>
       </c>
       <c r="I17" s="54"/>
@@ -16966,16 +17024,16 @@
       <c r="A18" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B18" s="118" t="s">
+      <c r="B18" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C18" s="119" t="s">
+      <c r="C18" s="118" t="s">
         <v>137</v>
       </c>
-      <c r="D18" s="120" t="s">
+      <c r="D18" s="119" t="s">
         <v>1044</v>
       </c>
-      <c r="E18" s="124">
+      <c r="E18" s="123">
         <v>0.74</v>
       </c>
       <c r="F18" s="93" t="s">
@@ -16984,7 +17042,7 @@
       <c r="G18" s="2" t="s">
         <v>1047</v>
       </c>
-      <c r="H18" s="122" t="s">
+      <c r="H18" s="121" t="s">
         <v>1045</v>
       </c>
       <c r="I18" s="54"/>
@@ -16993,16 +17051,16 @@
       <c r="A19" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B19" s="118" t="s">
+      <c r="B19" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C19" s="119" t="s">
+      <c r="C19" s="118" t="s">
         <v>137</v>
       </c>
-      <c r="D19" s="120" t="s">
+      <c r="D19" s="119" t="s">
         <v>1044</v>
       </c>
-      <c r="E19" s="124">
+      <c r="E19" s="123">
         <v>0.96</v>
       </c>
       <c r="F19" s="93" t="s">
@@ -17011,7 +17069,7 @@
       <c r="G19" s="2" t="s">
         <v>1049</v>
       </c>
-      <c r="H19" s="104" t="s">
+      <c r="H19" s="103" t="s">
         <v>1048</v>
       </c>
     </row>
@@ -17019,16 +17077,16 @@
       <c r="A20" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B20" s="118" t="s">
+      <c r="B20" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C20" s="119" t="s">
+      <c r="C20" s="118" t="s">
         <v>80</v>
       </c>
-      <c r="D20" s="120" t="s">
+      <c r="D20" s="119" t="s">
         <v>1044</v>
       </c>
-      <c r="E20" s="128">
+      <c r="E20" s="127">
         <v>1</v>
       </c>
       <c r="F20" s="93" t="s">
@@ -17037,7 +17095,7 @@
       <c r="G20" s="2" t="s">
         <v>1051</v>
       </c>
-      <c r="H20" s="104" t="s">
+      <c r="H20" s="103" t="s">
         <v>1050</v>
       </c>
     </row>
@@ -17045,16 +17103,16 @@
       <c r="A21" s="53" t="s">
         <v>1005</v>
       </c>
-      <c r="B21" s="118" t="s">
+      <c r="B21" s="117" t="s">
         <v>1006</v>
       </c>
-      <c r="C21" s="119" t="s">
+      <c r="C21" s="118" t="s">
         <v>135</v>
       </c>
-      <c r="D21" s="120" t="s">
+      <c r="D21" s="119" t="s">
         <v>1044</v>
       </c>
-      <c r="E21" s="121">
+      <c r="E21" s="120">
         <v>0.96</v>
       </c>
       <c r="F21" s="93" t="s">
@@ -17063,10 +17121,10 @@
       <c r="G21" s="2" t="s">
         <v>1051</v>
       </c>
-      <c r="H21" s="104" t="s">
+      <c r="H21" s="103" t="s">
         <v>1050</v>
       </c>
-      <c r="I21" s="123"/>
+      <c r="I21" s="122"/>
     </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
@@ -18587,19 +18645,19 @@
       <c r="B1" s="60" t="s">
         <v>926</v>
       </c>
-      <c r="C1" s="150" t="s">
+      <c r="C1" s="153" t="s">
         <v>167</v>
       </c>
-      <c r="D1" s="150"/>
+      <c r="D1" s="153"/>
       <c r="E1" s="61" t="s">
         <v>927</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="151" t="s">
+      <c r="A2" s="154" t="s">
         <v>932</v>
       </c>
-      <c r="B2" s="152" t="s">
+      <c r="B2" s="155" t="s">
         <v>933</v>
       </c>
       <c r="C2" s="26" t="s">
@@ -18610,8 +18668,8 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="151"/>
-      <c r="B3" s="152"/>
+      <c r="A3" s="154"/>
+      <c r="B3" s="155"/>
       <c r="C3" s="63" t="s">
         <v>936</v>
       </c>
@@ -18620,8 +18678,8 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="151"/>
-      <c r="B4" s="152"/>
+      <c r="A4" s="154"/>
+      <c r="B4" s="155"/>
       <c r="C4" s="65" t="s">
         <v>938</v>
       </c>
@@ -18630,8 +18688,8 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="151"/>
-      <c r="B5" s="152"/>
+      <c r="A5" s="154"/>
+      <c r="B5" s="155"/>
       <c r="C5" s="65" t="s">
         <v>940</v>
       </c>
@@ -18640,8 +18698,8 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="151"/>
-      <c r="B6" s="152"/>
+      <c r="A6" s="154"/>
+      <c r="B6" s="155"/>
       <c r="C6" s="28" t="s">
         <v>942</v>
       </c>
@@ -18650,8 +18708,8 @@
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="151"/>
-      <c r="B7" s="152"/>
+      <c r="A7" s="154"/>
+      <c r="B7" s="155"/>
       <c r="C7" s="68" t="s">
         <v>944</v>
       </c>
@@ -18660,7 +18718,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="151"/>
+      <c r="A8" s="154"/>
       <c r="B8" s="70" t="s">
         <v>946</v>
       </c>
@@ -18672,8 +18730,8 @@
       </c>
     </row>
     <row r="9" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="151"/>
-      <c r="B9" s="152" t="s">
+      <c r="A9" s="154"/>
+      <c r="B9" s="155" t="s">
         <v>949</v>
       </c>
       <c r="C9" s="72" t="s">
@@ -18685,8 +18743,8 @@
       <c r="E9" s="74"/>
     </row>
     <row r="10" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="151"/>
-      <c r="B10" s="152"/>
+      <c r="A10" s="154"/>
+      <c r="B10" s="155"/>
       <c r="C10" s="52" t="s">
         <v>952</v>
       </c>
@@ -18696,8 +18754,8 @@
       <c r="E10" s="74"/>
     </row>
     <row r="11" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="151"/>
-      <c r="B11" s="152"/>
+      <c r="A11" s="154"/>
+      <c r="B11" s="155"/>
       <c r="C11" s="52" t="s">
         <v>954</v>
       </c>
@@ -18707,8 +18765,8 @@
       <c r="E11" s="74"/>
     </row>
     <row r="12" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="151"/>
-      <c r="B12" s="152"/>
+      <c r="A12" s="154"/>
+      <c r="B12" s="155"/>
       <c r="C12" s="52" t="s">
         <v>956</v>
       </c>
@@ -18718,8 +18776,8 @@
       <c r="E12" s="74"/>
     </row>
     <row r="13" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="151"/>
-      <c r="B13" s="152"/>
+      <c r="A13" s="154"/>
+      <c r="B13" s="155"/>
       <c r="C13" s="52" t="s">
         <v>958</v>
       </c>
@@ -18729,8 +18787,8 @@
       <c r="E13" s="74"/>
     </row>
     <row r="14" spans="1:5" s="14" customFormat="1" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="151"/>
-      <c r="B14" s="152"/>
+      <c r="A14" s="154"/>
+      <c r="B14" s="155"/>
       <c r="C14" s="52" t="s">
         <v>959</v>
       </c>
@@ -18740,8 +18798,8 @@
       <c r="E14" s="74"/>
     </row>
     <row r="15" spans="1:5" s="14" customFormat="1" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="151"/>
-      <c r="B15" s="152"/>
+      <c r="A15" s="154"/>
+      <c r="B15" s="155"/>
       <c r="C15" s="77" t="s">
         <v>961</v>
       </c>
@@ -18751,10 +18809,10 @@
       <c r="E15" s="74"/>
     </row>
     <row r="16" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="153" t="s">
+      <c r="A16" s="156" t="s">
         <v>963</v>
       </c>
-      <c r="B16" s="154" t="s">
+      <c r="B16" s="157" t="s">
         <v>964</v>
       </c>
       <c r="C16" s="72" t="s">
@@ -18768,8 +18826,8 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="153"/>
-      <c r="B17" s="154"/>
+      <c r="A17" s="156"/>
+      <c r="B17" s="157"/>
       <c r="C17" s="28" t="s">
         <v>966</v>
       </c>
@@ -18781,8 +18839,8 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="153"/>
-      <c r="B18" s="149" t="s">
+      <c r="A18" s="156"/>
+      <c r="B18" s="152" t="s">
         <v>968</v>
       </c>
       <c r="C18" s="26" t="s">
@@ -18796,8 +18854,8 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="153"/>
-      <c r="B19" s="149"/>
+      <c r="A19" s="156"/>
+      <c r="B19" s="152"/>
       <c r="C19" s="28" t="s">
         <v>970</v>
       </c>
@@ -18809,10 +18867,10 @@
       </c>
     </row>
     <row r="20" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="147" t="s">
+      <c r="A20" s="150" t="s">
         <v>973</v>
       </c>
-      <c r="B20" s="148" t="s">
+      <c r="B20" s="151" t="s">
         <v>974</v>
       </c>
       <c r="C20" s="81" t="s">
@@ -18823,8 +18881,8 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="147"/>
-      <c r="B21" s="147"/>
+      <c r="A21" s="150"/>
+      <c r="B21" s="150"/>
       <c r="C21" s="9" t="s">
         <v>977</v>
       </c>
@@ -18833,8 +18891,8 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="147"/>
-      <c r="B22" s="147"/>
+      <c r="A22" s="150"/>
+      <c r="B22" s="150"/>
       <c r="C22" s="9" t="s">
         <v>923</v>
       </c>
@@ -18843,8 +18901,8 @@
       </c>
     </row>
     <row r="23" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="147"/>
-      <c r="B23" s="147"/>
+      <c r="A23" s="150"/>
+      <c r="B23" s="150"/>
       <c r="C23" s="84" t="s">
         <v>979</v>
       </c>
@@ -18853,8 +18911,8 @@
       </c>
     </row>
     <row r="24" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="147"/>
-      <c r="B24" s="148"/>
+      <c r="A24" s="150"/>
+      <c r="B24" s="151"/>
       <c r="C24" s="22" t="s">
         <v>980</v>
       </c>
@@ -18863,8 +18921,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="147"/>
-      <c r="B25" s="149" t="s">
+      <c r="A25" s="150"/>
+      <c r="B25" s="152" t="s">
         <v>982</v>
       </c>
       <c r="C25" s="87" t="s">
@@ -18875,8 +18933,8 @@
       </c>
     </row>
     <row r="26" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="147"/>
-      <c r="B26" s="149"/>
+      <c r="A26" s="150"/>
+      <c r="B26" s="152"/>
       <c r="C26" s="89" t="s">
         <v>985</v>
       </c>
@@ -19420,10 +19478,10 @@
       <c r="A2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="116">
+      <c r="B2" s="115">
         <v>0.74</v>
       </c>
-      <c r="C2" s="116">
+      <c r="C2" s="115">
         <v>0.81</v>
       </c>
       <c r="D2" s="99"/>
@@ -19543,10 +19601,10 @@
       <c r="A5" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B5" s="117">
+      <c r="B5" s="116">
         <v>0.9</v>
       </c>
-      <c r="C5" s="117">
+      <c r="C5" s="116">
         <v>0.9</v>
       </c>
       <c r="D5" s="99"/>
@@ -19585,7 +19643,7 @@
         <v>88</v>
       </c>
       <c r="B6" s="16"/>
-      <c r="C6" s="108"/>
+      <c r="C6" s="107"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
@@ -19621,10 +19679,10 @@
       <c r="A7" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="117">
+      <c r="B7" s="116">
         <v>0</v>
       </c>
-      <c r="C7" s="117">
+      <c r="C7" s="116">
         <v>0</v>
       </c>
       <c r="D7" s="99"/>
@@ -19662,10 +19720,10 @@
       <c r="A8" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="116">
+      <c r="B8" s="115">
         <v>0.95</v>
       </c>
-      <c r="C8" s="116">
+      <c r="C8" s="115">
         <v>0.95</v>
       </c>
       <c r="D8" s="99"/>
@@ -19704,7 +19762,7 @@
         <v>93</v>
       </c>
       <c r="B9" s="16"/>
-      <c r="C9" s="108"/>
+      <c r="C9" s="107"/>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
       <c r="F9" s="3"/>
@@ -19741,7 +19799,7 @@
         <v>95</v>
       </c>
       <c r="B10" s="16"/>
-      <c r="C10" s="108"/>
+      <c r="C10" s="107"/>
       <c r="D10" s="3"/>
       <c r="E10" s="99"/>
       <c r="F10" s="3"/>
@@ -19778,7 +19836,7 @@
         <v>97</v>
       </c>
       <c r="B11" s="16"/>
-      <c r="C11" s="108"/>
+      <c r="C11" s="107"/>
       <c r="D11" s="3"/>
       <c r="E11" s="3"/>
       <c r="F11" s="99"/>
@@ -19814,10 +19872,10 @@
       <c r="A12" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="116">
+      <c r="B12" s="115">
         <v>0.95</v>
       </c>
-      <c r="C12" s="116">
+      <c r="C12" s="115">
         <v>0.95</v>
       </c>
       <c r="D12" s="99"/>
@@ -19856,7 +19914,7 @@
         <v>100</v>
       </c>
       <c r="B13" s="16"/>
-      <c r="C13" s="108"/>
+      <c r="C13" s="107"/>
       <c r="D13" s="3"/>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
@@ -19893,7 +19951,7 @@
         <v>102</v>
       </c>
       <c r="B14" s="16"/>
-      <c r="C14" s="108"/>
+      <c r="C14" s="107"/>
       <c r="D14" s="3"/>
       <c r="E14" s="99"/>
       <c r="F14" s="99"/>
@@ -19929,10 +19987,10 @@
       <c r="A15" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="B15" s="117">
+      <c r="B15" s="116">
         <v>0.9</v>
       </c>
-      <c r="C15" s="117">
+      <c r="C15" s="116">
         <v>0.9</v>
       </c>
       <c r="D15" s="99"/>
@@ -19970,10 +20028,10 @@
       <c r="A16" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="116">
+      <c r="B16" s="115">
         <v>0</v>
       </c>
-      <c r="C16" s="116">
+      <c r="C16" s="115">
         <v>0.98</v>
       </c>
       <c r="D16" s="99"/>
@@ -20012,7 +20070,7 @@
         <v>112</v>
       </c>
       <c r="B17" s="16"/>
-      <c r="C17" s="108"/>
+      <c r="C17" s="107"/>
       <c r="D17" s="3"/>
       <c r="E17" s="3"/>
       <c r="F17" s="3"/>
@@ -20049,7 +20107,7 @@
         <v>114</v>
       </c>
       <c r="B18" s="16"/>
-      <c r="C18" s="108"/>
+      <c r="C18" s="107"/>
       <c r="D18" s="3"/>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
@@ -20086,7 +20144,7 @@
         <v>116</v>
       </c>
       <c r="B19" s="16"/>
-      <c r="C19" s="108"/>
+      <c r="C19" s="107"/>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
@@ -20122,10 +20180,10 @@
       <c r="A20" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="B20" s="117">
+      <c r="B20" s="116">
         <v>0.9</v>
       </c>
-      <c r="C20" s="117">
+      <c r="C20" s="116">
         <v>0.9</v>
       </c>
       <c r="D20" s="99"/>
@@ -20164,7 +20222,7 @@
         <v>120</v>
       </c>
       <c r="B21" s="16"/>
-      <c r="C21" s="108"/>
+      <c r="C21" s="107"/>
       <c r="D21" s="3"/>
       <c r="E21" s="3"/>
       <c r="F21" s="3"/>
@@ -20200,10 +20258,10 @@
       <c r="A22" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B22" s="117">
+      <c r="B22" s="116">
         <v>0.9</v>
       </c>
-      <c r="C22" s="117">
+      <c r="C22" s="116">
         <v>0.9</v>
       </c>
       <c r="D22" s="99"/>
@@ -20242,7 +20300,7 @@
         <v>124</v>
       </c>
       <c r="B23" s="16"/>
-      <c r="C23" s="108"/>
+      <c r="C23" s="107"/>
       <c r="D23" s="3"/>
       <c r="E23" s="3"/>
       <c r="F23" s="3"/>
@@ -20278,10 +20336,10 @@
       <c r="A24" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="B24" s="116">
+      <c r="B24" s="115">
         <v>0</v>
       </c>
-      <c r="C24" s="116">
+      <c r="C24" s="115">
         <v>0</v>
       </c>
       <c r="D24" s="99"/>
@@ -20320,7 +20378,7 @@
         <v>129</v>
       </c>
       <c r="B25" s="16"/>
-      <c r="C25" s="108"/>
+      <c r="C25" s="107"/>
       <c r="D25" s="3"/>
       <c r="E25" s="3"/>
       <c r="F25" s="3"/>
@@ -20393,10 +20451,10 @@
       <c r="A27" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B27" s="116">
+      <c r="B27" s="115">
         <v>0</v>
       </c>
-      <c r="C27" s="116">
+      <c r="C27" s="115">
         <v>0</v>
       </c>
       <c r="D27" s="3"/>
@@ -20434,10 +20492,10 @@
       <c r="A28" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B28" s="116">
+      <c r="B28" s="115">
         <v>0</v>
       </c>
-      <c r="C28" s="116">
+      <c r="C28" s="115">
         <v>0</v>
       </c>
       <c r="D28" s="3"/>
@@ -20586,10 +20644,10 @@
       <c r="A32" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="116">
+      <c r="B32" s="115">
         <v>0</v>
       </c>
-      <c r="C32" s="116">
+      <c r="C32" s="115">
         <v>0</v>
       </c>
       <c r="D32" s="99"/>
@@ -20665,7 +20723,7 @@
         <v>151</v>
       </c>
       <c r="B34" s="3"/>
-      <c r="C34" s="108"/>
+      <c r="C34" s="107"/>
       <c r="D34" s="3"/>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
@@ -20702,7 +20760,7 @@
         <v>153</v>
       </c>
       <c r="B35" s="3"/>
-      <c r="C35" s="108"/>
+      <c r="C35" s="107"/>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
@@ -20738,10 +20796,10 @@
       <c r="A36" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="B36" s="117">
+      <c r="B36" s="116">
         <v>0.9</v>
       </c>
-      <c r="C36" s="117">
+      <c r="C36" s="116">
         <v>0.9</v>
       </c>
       <c r="D36" s="99"/>
@@ -20780,7 +20838,7 @@
         <v>157</v>
       </c>
       <c r="B37" s="3"/>
-      <c r="C37" s="108"/>
+      <c r="C37" s="107"/>
       <c r="D37" s="3"/>
       <c r="E37" s="3"/>
       <c r="F37" s="3"/>
@@ -20817,7 +20875,7 @@
         <v>131</v>
       </c>
       <c r="B38" s="3"/>
-      <c r="C38" s="108"/>
+      <c r="C38" s="107"/>
       <c r="D38" s="3"/>
       <c r="E38" s="3"/>
       <c r="F38" s="3"/>
@@ -22127,452 +22185,944 @@
       <c r="A2" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="B2" s="103"/>
-      <c r="C2" s="103"/>
-      <c r="D2" s="103"/>
-      <c r="E2" s="103"/>
-      <c r="F2" s="103"/>
-      <c r="G2" s="103"/>
+      <c r="B2" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C2" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D2" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E2" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F2" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G2" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="B3" s="103"/>
-      <c r="C3" s="103"/>
-      <c r="D3" s="103"/>
-      <c r="E3" s="103"/>
-      <c r="F3" s="103"/>
-      <c r="G3" s="103"/>
+      <c r="B3" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C3" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D3" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E3" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F3" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G3" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="B4" s="103"/>
-      <c r="C4" s="103"/>
-      <c r="D4" s="103"/>
-      <c r="E4" s="103"/>
-      <c r="F4" s="103"/>
-      <c r="G4" s="103"/>
+      <c r="B4" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C4" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D4" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E4" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F4" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G4" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B5" s="103"/>
-      <c r="C5" s="103"/>
-      <c r="D5" s="103"/>
-      <c r="E5" s="103"/>
-      <c r="F5" s="103"/>
-      <c r="G5" s="103"/>
+      <c r="B5" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C5" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D5" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E5" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F5" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G5" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="B6" s="103"/>
-      <c r="C6" s="103"/>
-      <c r="D6" s="103"/>
-      <c r="E6" s="103"/>
-      <c r="F6" s="103"/>
-      <c r="G6" s="103"/>
+      <c r="B6" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C6" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D6" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E6" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F6" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G6" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B7" s="103"/>
-      <c r="C7" s="103"/>
-      <c r="D7" s="103"/>
-      <c r="E7" s="103"/>
-      <c r="F7" s="103"/>
-      <c r="G7" s="103"/>
+      <c r="B7" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C7" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D7" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E7" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F7" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G7" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="B8" s="103"/>
-      <c r="C8" s="103"/>
-      <c r="D8" s="103"/>
-      <c r="E8" s="103"/>
-      <c r="F8" s="103"/>
-      <c r="G8" s="103"/>
+      <c r="B8" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C8" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D8" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E8" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F8" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="B9" s="103"/>
-      <c r="C9" s="103"/>
-      <c r="D9" s="103"/>
-      <c r="E9" s="103"/>
-      <c r="F9" s="103"/>
-      <c r="G9" s="103"/>
+      <c r="B9" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C9" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D9" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E9" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F9" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G9" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B10" s="103"/>
-      <c r="C10" s="103"/>
-      <c r="D10" s="103"/>
-      <c r="E10" s="103"/>
-      <c r="F10" s="103"/>
-      <c r="G10" s="103"/>
+      <c r="B10" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C10" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D10" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E10" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F10" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G10" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="B11" s="103"/>
-      <c r="C11" s="103"/>
-      <c r="D11" s="103"/>
-      <c r="E11" s="103"/>
-      <c r="F11" s="103"/>
-      <c r="G11" s="103"/>
+      <c r="B11" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C11" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D11" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E11" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F11" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G11" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="B12" s="103"/>
-      <c r="C12" s="103"/>
-      <c r="D12" s="103"/>
-      <c r="E12" s="103"/>
-      <c r="F12" s="103"/>
-      <c r="G12" s="103"/>
+      <c r="B12" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C12" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D12" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F12" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G12" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="B13" s="103"/>
-      <c r="C13" s="103"/>
-      <c r="D13" s="103"/>
-      <c r="E13" s="103"/>
-      <c r="F13" s="103"/>
-      <c r="G13" s="103"/>
+      <c r="B13" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C13" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D13" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E13" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F13" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G13" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="B14" s="103"/>
-      <c r="C14" s="103"/>
-      <c r="D14" s="103"/>
-      <c r="E14" s="103"/>
-      <c r="F14" s="103"/>
-      <c r="G14" s="103"/>
+      <c r="B14" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C14" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D14" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E14" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F14" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G14" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="B15" s="103"/>
-      <c r="C15" s="103"/>
-      <c r="D15" s="103"/>
-      <c r="E15" s="103"/>
-      <c r="F15" s="103"/>
-      <c r="G15" s="103"/>
+      <c r="B15" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C15" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D15" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E15" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F15" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G15" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B16" s="103"/>
-      <c r="C16" s="103"/>
-      <c r="D16" s="103"/>
-      <c r="E16" s="103"/>
-      <c r="F16" s="103"/>
-      <c r="G16" s="103"/>
+      <c r="B16" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C16" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D16" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E16" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F16" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G16" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B17" s="103"/>
-      <c r="C17" s="103"/>
-      <c r="D17" s="103"/>
-      <c r="E17" s="103"/>
-      <c r="F17" s="103"/>
-      <c r="G17" s="103"/>
+      <c r="B17" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C17" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D17" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E17" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F17" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G17" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="B18" s="103"/>
-      <c r="C18" s="103"/>
-      <c r="D18" s="103"/>
-      <c r="E18" s="103"/>
-      <c r="F18" s="103"/>
-      <c r="G18" s="103"/>
+      <c r="B18" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C18" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D18" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E18" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F18" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G18" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="B19" s="103"/>
-      <c r="C19" s="103"/>
-      <c r="D19" s="103"/>
-      <c r="E19" s="103"/>
-      <c r="F19" s="103"/>
-      <c r="G19" s="103"/>
+      <c r="B19" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C19" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D19" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E19" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F19" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G19" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="B20" s="103"/>
-      <c r="C20" s="103"/>
-      <c r="D20" s="103"/>
-      <c r="E20" s="103"/>
-      <c r="F20" s="103"/>
-      <c r="G20" s="103"/>
+      <c r="B20" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C20" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D20" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E20" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F20" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G20" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B21" s="103"/>
-      <c r="C21" s="103"/>
-      <c r="D21" s="103"/>
-      <c r="E21" s="103"/>
-      <c r="F21" s="103"/>
-      <c r="G21" s="103"/>
+      <c r="B21" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C21" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D21" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E21" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F21" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G21" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B22" s="103"/>
-      <c r="C22" s="103"/>
-      <c r="D22" s="103"/>
-      <c r="E22" s="103"/>
-      <c r="F22" s="103"/>
-      <c r="G22" s="103"/>
+      <c r="B22" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C22" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D22" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E22" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F22" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G22" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="B23" s="103"/>
-      <c r="C23" s="103"/>
-      <c r="D23" s="103"/>
-      <c r="E23" s="103"/>
-      <c r="F23" s="103"/>
-      <c r="G23" s="103"/>
+      <c r="B23" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C23" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D23" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E23" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F23" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G23" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="B24" s="103"/>
-      <c r="C24" s="103"/>
-      <c r="D24" s="103"/>
-      <c r="E24" s="103"/>
-      <c r="F24" s="103"/>
-      <c r="G24" s="103"/>
+      <c r="B24" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C24" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D24" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E24" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F24" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G24" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="B25" s="103"/>
-      <c r="C25" s="103"/>
-      <c r="D25" s="103"/>
-      <c r="E25" s="103"/>
-      <c r="F25" s="103"/>
-      <c r="G25" s="103"/>
+      <c r="B25" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C25" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D25" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E25" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F25" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G25" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="B26" s="103"/>
-      <c r="C26" s="103"/>
-      <c r="D26" s="103"/>
-      <c r="E26" s="103"/>
-      <c r="F26" s="103"/>
-      <c r="G26" s="103"/>
+      <c r="B26" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C26" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D26" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E26" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F26" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G26" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B27" s="103"/>
-      <c r="C27" s="103"/>
-      <c r="D27" s="103"/>
-      <c r="E27" s="103"/>
-      <c r="F27" s="103"/>
-      <c r="G27" s="103"/>
+      <c r="B27" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C27" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D27" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E27" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F27" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G27" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B28" s="103"/>
-      <c r="C28" s="103"/>
-      <c r="D28" s="103"/>
-      <c r="E28" s="103"/>
-      <c r="F28" s="103"/>
-      <c r="G28" s="103"/>
+      <c r="B28" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C28" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D28" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E28" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F28" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G28" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="B29" s="103"/>
-      <c r="C29" s="103"/>
-      <c r="D29" s="103"/>
-      <c r="E29" s="103"/>
-      <c r="F29" s="103"/>
-      <c r="G29" s="103"/>
+      <c r="B29" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C29" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D29" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E29" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F29" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G29" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="B30" s="103"/>
-      <c r="C30" s="103"/>
-      <c r="D30" s="103"/>
-      <c r="E30" s="103"/>
-      <c r="F30" s="103"/>
-      <c r="G30" s="103"/>
+      <c r="B30" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C30" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D30" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E30" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F30" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G30" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B31" s="103"/>
-      <c r="C31" s="103"/>
-      <c r="D31" s="103"/>
-      <c r="E31" s="103"/>
-      <c r="F31" s="103"/>
-      <c r="G31" s="103"/>
+      <c r="B31" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C31" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D31" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E31" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F31" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G31" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B32" s="103"/>
-      <c r="C32" s="103"/>
-      <c r="D32" s="103"/>
-      <c r="E32" s="103"/>
-      <c r="F32" s="103"/>
-      <c r="G32" s="103"/>
+      <c r="B32" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C32" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D32" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E32" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F32" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G32" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B33" s="103"/>
-      <c r="C33" s="103"/>
-      <c r="D33" s="103"/>
-      <c r="E33" s="103"/>
-      <c r="F33" s="103"/>
-      <c r="G33" s="103"/>
+      <c r="B33" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C33" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D33" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E33" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F33" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G33" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="B34" s="103"/>
-      <c r="C34" s="103"/>
-      <c r="D34" s="103"/>
-      <c r="E34" s="103"/>
-      <c r="F34" s="103"/>
-      <c r="G34" s="103"/>
+      <c r="B34" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C34" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D34" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E34" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F34" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G34" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="B35" s="103"/>
-      <c r="C35" s="103"/>
-      <c r="D35" s="103"/>
-      <c r="E35" s="103"/>
-      <c r="F35" s="103"/>
-      <c r="G35" s="103"/>
+      <c r="B35" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C35" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D35" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E35" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F35" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G35" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="B36" s="103"/>
-      <c r="C36" s="103"/>
-      <c r="D36" s="103"/>
-      <c r="E36" s="103"/>
-      <c r="F36" s="103"/>
-      <c r="G36" s="103"/>
+      <c r="B36" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C36" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D36" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E36" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F36" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G36" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="B37" s="103"/>
-      <c r="C37" s="103"/>
-      <c r="D37" s="103"/>
-      <c r="E37" s="103"/>
-      <c r="F37" s="103"/>
-      <c r="G37" s="103"/>
+      <c r="B37" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C37" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D37" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E37" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F37" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G37" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B38" s="103"/>
-      <c r="C38" s="103"/>
-      <c r="D38" s="103"/>
-      <c r="E38" s="103"/>
-      <c r="F38" s="103"/>
-      <c r="G38" s="103"/>
+      <c r="B38" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C38" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D38" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E38" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F38" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G38" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B39" s="103"/>
-      <c r="C39" s="103"/>
-      <c r="D39" s="103"/>
-      <c r="E39" s="103"/>
-      <c r="F39" s="103"/>
-      <c r="G39" s="103"/>
+      <c r="B39" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C39" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D39" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E39" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F39" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G39" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B40" s="103"/>
-      <c r="C40" s="103"/>
-      <c r="D40" s="103"/>
-      <c r="E40" s="103"/>
-      <c r="F40" s="103"/>
-      <c r="G40" s="103"/>
+      <c r="B40" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C40" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D40" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E40" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F40" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G40" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B41" s="103"/>
-      <c r="C41" s="103"/>
-      <c r="D41" s="103"/>
-      <c r="E41" s="103"/>
-      <c r="F41" s="103"/>
-      <c r="G41" s="103"/>
+      <c r="B41" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C41" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D41" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E41" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F41" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G41" s="129">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B42" s="103"/>
-      <c r="C42" s="103"/>
-      <c r="D42" s="103"/>
-      <c r="E42" s="103"/>
-      <c r="F42" s="103"/>
-      <c r="G42" s="103"/>
+      <c r="B42" s="129">
+        <v>0.1</v>
+      </c>
+      <c r="C42" s="129">
+        <v>0.2</v>
+      </c>
+      <c r="D42" s="129">
+        <v>0.3</v>
+      </c>
+      <c r="E42" s="129">
+        <v>0.4</v>
+      </c>
+      <c r="F42" s="129">
+        <v>0.5</v>
+      </c>
+      <c r="G42" s="129">
+        <v>0.7</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -22582,7 +23132,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30748705-90F8-C045-BB2B-8F50A72C1112}">
   <sheetPr>
-    <tabColor rgb="FF002060"/>
+    <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -22617,22 +23167,22 @@
       <c r="A2" s="21" t="s">
         <v>1056</v>
       </c>
-      <c r="B2" s="155">
+      <c r="B2" s="129">
         <v>0.9</v>
       </c>
-      <c r="C2" s="155">
+      <c r="C2" s="129">
         <v>0.9</v>
       </c>
-      <c r="D2" s="155">
+      <c r="D2" s="129">
         <v>0.9</v>
       </c>
-      <c r="E2" s="155">
+      <c r="E2" s="129">
         <v>0.9</v>
       </c>
-      <c r="F2" s="155">
+      <c r="F2" s="129">
         <v>0.9</v>
       </c>
-      <c r="G2" s="155">
+      <c r="G2" s="129">
         <v>0.9</v>
       </c>
     </row>
@@ -22640,22 +23190,22 @@
       <c r="A3" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="155">
+      <c r="B3" s="129">
         <v>0.15</v>
       </c>
-      <c r="C3" s="155">
+      <c r="C3" s="129">
         <v>0.3</v>
       </c>
-      <c r="D3" s="155">
+      <c r="D3" s="129">
         <v>0.4</v>
       </c>
-      <c r="E3" s="155">
+      <c r="E3" s="129">
         <v>0.5</v>
       </c>
-      <c r="F3" s="155">
+      <c r="F3" s="129">
         <v>0.6</v>
       </c>
-      <c r="G3" s="155">
+      <c r="G3" s="129">
         <v>0.7</v>
       </c>
     </row>
@@ -22663,366 +23213,366 @@
       <c r="A4" s="21" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="155">
+      <c r="B4" s="129">
         <v>0.15</v>
       </c>
-      <c r="C4" s="155">
+      <c r="C4" s="129">
         <v>0.3</v>
       </c>
-      <c r="D4" s="155">
+      <c r="D4" s="129">
         <v>0.4</v>
       </c>
-      <c r="E4" s="155">
+      <c r="E4" s="129">
         <v>0.5</v>
       </c>
-      <c r="F4" s="155">
+      <c r="F4" s="129">
         <v>0.6</v>
       </c>
-      <c r="G4" s="155">
+      <c r="G4" s="129">
         <v>0.7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="21"/>
-      <c r="B5" s="155"/>
-      <c r="C5" s="155"/>
-      <c r="D5" s="155"/>
-      <c r="E5" s="155"/>
-      <c r="F5" s="155"/>
-      <c r="G5" s="155"/>
+      <c r="B5" s="129"/>
+      <c r="C5" s="129"/>
+      <c r="D5" s="129"/>
+      <c r="E5" s="129"/>
+      <c r="F5" s="129"/>
+      <c r="G5" s="129"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="21"/>
-      <c r="B6" s="155"/>
-      <c r="C6" s="155"/>
-      <c r="D6" s="155"/>
-      <c r="E6" s="155"/>
-      <c r="F6" s="155"/>
-      <c r="G6" s="155"/>
+      <c r="B6" s="129"/>
+      <c r="C6" s="129"/>
+      <c r="D6" s="129"/>
+      <c r="E6" s="129"/>
+      <c r="F6" s="129"/>
+      <c r="G6" s="129"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="21"/>
-      <c r="B7" s="155"/>
-      <c r="C7" s="155"/>
-      <c r="D7" s="155"/>
-      <c r="E7" s="155"/>
-      <c r="F7" s="155"/>
-      <c r="G7" s="155"/>
+      <c r="B7" s="129"/>
+      <c r="C7" s="129"/>
+      <c r="D7" s="129"/>
+      <c r="E7" s="129"/>
+      <c r="F7" s="129"/>
+      <c r="G7" s="129"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="21"/>
-      <c r="B8" s="155"/>
-      <c r="C8" s="155"/>
-      <c r="D8" s="155"/>
-      <c r="E8" s="155"/>
-      <c r="F8" s="155"/>
-      <c r="G8" s="155"/>
+      <c r="B8" s="129"/>
+      <c r="C8" s="129"/>
+      <c r="D8" s="129"/>
+      <c r="E8" s="129"/>
+      <c r="F8" s="129"/>
+      <c r="G8" s="129"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="21"/>
-      <c r="B9" s="155"/>
-      <c r="C9" s="155"/>
-      <c r="D9" s="155"/>
-      <c r="E9" s="155"/>
-      <c r="F9" s="155"/>
-      <c r="G9" s="155"/>
+      <c r="B9" s="129"/>
+      <c r="C9" s="129"/>
+      <c r="D9" s="129"/>
+      <c r="E9" s="129"/>
+      <c r="F9" s="129"/>
+      <c r="G9" s="129"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" s="21"/>
-      <c r="B10" s="155"/>
-      <c r="C10" s="155"/>
-      <c r="D10" s="155"/>
-      <c r="E10" s="155"/>
-      <c r="F10" s="155"/>
-      <c r="G10" s="155"/>
+      <c r="B10" s="129"/>
+      <c r="C10" s="129"/>
+      <c r="D10" s="129"/>
+      <c r="E10" s="129"/>
+      <c r="F10" s="129"/>
+      <c r="G10" s="129"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="21"/>
-      <c r="B11" s="155"/>
-      <c r="C11" s="155"/>
-      <c r="D11" s="155"/>
-      <c r="E11" s="155"/>
-      <c r="F11" s="155"/>
-      <c r="G11" s="155"/>
+      <c r="B11" s="129"/>
+      <c r="C11" s="129"/>
+      <c r="D11" s="129"/>
+      <c r="E11" s="129"/>
+      <c r="F11" s="129"/>
+      <c r="G11" s="129"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="21"/>
-      <c r="B12" s="155"/>
-      <c r="C12" s="155"/>
-      <c r="D12" s="155"/>
-      <c r="E12" s="155"/>
-      <c r="F12" s="155"/>
-      <c r="G12" s="155"/>
+      <c r="B12" s="129"/>
+      <c r="C12" s="129"/>
+      <c r="D12" s="129"/>
+      <c r="E12" s="129"/>
+      <c r="F12" s="129"/>
+      <c r="G12" s="129"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="21"/>
-      <c r="B13" s="155"/>
-      <c r="C13" s="155"/>
-      <c r="D13" s="155"/>
-      <c r="E13" s="155"/>
-      <c r="F13" s="155"/>
-      <c r="G13" s="155"/>
+      <c r="B13" s="129"/>
+      <c r="C13" s="129"/>
+      <c r="D13" s="129"/>
+      <c r="E13" s="129"/>
+      <c r="F13" s="129"/>
+      <c r="G13" s="129"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="21"/>
-      <c r="B14" s="155"/>
-      <c r="C14" s="155"/>
-      <c r="D14" s="155"/>
-      <c r="E14" s="155"/>
-      <c r="F14" s="155"/>
-      <c r="G14" s="155"/>
+      <c r="B14" s="129"/>
+      <c r="C14" s="129"/>
+      <c r="D14" s="129"/>
+      <c r="E14" s="129"/>
+      <c r="F14" s="129"/>
+      <c r="G14" s="129"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="21"/>
-      <c r="B15" s="155"/>
-      <c r="C15" s="155"/>
-      <c r="D15" s="155"/>
-      <c r="E15" s="155"/>
-      <c r="F15" s="155"/>
-      <c r="G15" s="155"/>
+      <c r="B15" s="129"/>
+      <c r="C15" s="129"/>
+      <c r="D15" s="129"/>
+      <c r="E15" s="129"/>
+      <c r="F15" s="129"/>
+      <c r="G15" s="129"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A16" s="21"/>
-      <c r="B16" s="155"/>
-      <c r="C16" s="155"/>
-      <c r="D16" s="155"/>
-      <c r="E16" s="155"/>
-      <c r="F16" s="155"/>
-      <c r="G16" s="155"/>
+      <c r="B16" s="129"/>
+      <c r="C16" s="129"/>
+      <c r="D16" s="129"/>
+      <c r="E16" s="129"/>
+      <c r="F16" s="129"/>
+      <c r="G16" s="129"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A17" s="21"/>
-      <c r="B17" s="155"/>
-      <c r="C17" s="155"/>
-      <c r="D17" s="155"/>
-      <c r="E17" s="155"/>
-      <c r="F17" s="155"/>
-      <c r="G17" s="155"/>
+      <c r="B17" s="129"/>
+      <c r="C17" s="129"/>
+      <c r="D17" s="129"/>
+      <c r="E17" s="129"/>
+      <c r="F17" s="129"/>
+      <c r="G17" s="129"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A18" s="21"/>
-      <c r="B18" s="155"/>
-      <c r="C18" s="155"/>
-      <c r="D18" s="155"/>
-      <c r="E18" s="155"/>
-      <c r="F18" s="155"/>
-      <c r="G18" s="155"/>
+      <c r="B18" s="129"/>
+      <c r="C18" s="129"/>
+      <c r="D18" s="129"/>
+      <c r="E18" s="129"/>
+      <c r="F18" s="129"/>
+      <c r="G18" s="129"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A19" s="21"/>
-      <c r="B19" s="155"/>
-      <c r="C19" s="155"/>
-      <c r="D19" s="155"/>
-      <c r="E19" s="155"/>
-      <c r="F19" s="155"/>
-      <c r="G19" s="155"/>
+      <c r="B19" s="129"/>
+      <c r="C19" s="129"/>
+      <c r="D19" s="129"/>
+      <c r="E19" s="129"/>
+      <c r="F19" s="129"/>
+      <c r="G19" s="129"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A20" s="21"/>
-      <c r="B20" s="155"/>
-      <c r="C20" s="155"/>
-      <c r="D20" s="155"/>
-      <c r="E20" s="155"/>
-      <c r="F20" s="155"/>
-      <c r="G20" s="155"/>
+      <c r="B20" s="129"/>
+      <c r="C20" s="129"/>
+      <c r="D20" s="129"/>
+      <c r="E20" s="129"/>
+      <c r="F20" s="129"/>
+      <c r="G20" s="129"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A21" s="21"/>
-      <c r="B21" s="155"/>
-      <c r="C21" s="155"/>
-      <c r="D21" s="155"/>
-      <c r="E21" s="155"/>
-      <c r="F21" s="155"/>
-      <c r="G21" s="155"/>
+      <c r="B21" s="129"/>
+      <c r="C21" s="129"/>
+      <c r="D21" s="129"/>
+      <c r="E21" s="129"/>
+      <c r="F21" s="129"/>
+      <c r="G21" s="129"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A22" s="21"/>
-      <c r="B22" s="155"/>
-      <c r="C22" s="155"/>
-      <c r="D22" s="155"/>
-      <c r="E22" s="155"/>
-      <c r="F22" s="155"/>
-      <c r="G22" s="155"/>
+      <c r="B22" s="129"/>
+      <c r="C22" s="129"/>
+      <c r="D22" s="129"/>
+      <c r="E22" s="129"/>
+      <c r="F22" s="129"/>
+      <c r="G22" s="129"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="21"/>
-      <c r="B23" s="155"/>
-      <c r="C23" s="155"/>
-      <c r="D23" s="155"/>
-      <c r="E23" s="155"/>
-      <c r="F23" s="155"/>
-      <c r="G23" s="155"/>
+      <c r="B23" s="129"/>
+      <c r="C23" s="129"/>
+      <c r="D23" s="129"/>
+      <c r="E23" s="129"/>
+      <c r="F23" s="129"/>
+      <c r="G23" s="129"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A24" s="21"/>
-      <c r="B24" s="155"/>
-      <c r="C24" s="155"/>
-      <c r="D24" s="155"/>
-      <c r="E24" s="155"/>
-      <c r="F24" s="155"/>
-      <c r="G24" s="155"/>
+      <c r="B24" s="129"/>
+      <c r="C24" s="129"/>
+      <c r="D24" s="129"/>
+      <c r="E24" s="129"/>
+      <c r="F24" s="129"/>
+      <c r="G24" s="129"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A25" s="21"/>
-      <c r="B25" s="155"/>
-      <c r="C25" s="155"/>
-      <c r="D25" s="155"/>
-      <c r="E25" s="155"/>
-      <c r="F25" s="155"/>
-      <c r="G25" s="155"/>
+      <c r="B25" s="129"/>
+      <c r="C25" s="129"/>
+      <c r="D25" s="129"/>
+      <c r="E25" s="129"/>
+      <c r="F25" s="129"/>
+      <c r="G25" s="129"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A26" s="21"/>
-      <c r="B26" s="155"/>
-      <c r="C26" s="155"/>
-      <c r="D26" s="155"/>
-      <c r="E26" s="155"/>
-      <c r="F26" s="155"/>
-      <c r="G26" s="155"/>
+      <c r="B26" s="129"/>
+      <c r="C26" s="129"/>
+      <c r="D26" s="129"/>
+      <c r="E26" s="129"/>
+      <c r="F26" s="129"/>
+      <c r="G26" s="129"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A27" s="21"/>
-      <c r="B27" s="155"/>
-      <c r="C27" s="155"/>
-      <c r="D27" s="155"/>
-      <c r="E27" s="155"/>
-      <c r="F27" s="155"/>
-      <c r="G27" s="155"/>
+      <c r="B27" s="129"/>
+      <c r="C27" s="129"/>
+      <c r="D27" s="129"/>
+      <c r="E27" s="129"/>
+      <c r="F27" s="129"/>
+      <c r="G27" s="129"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A28" s="21"/>
-      <c r="B28" s="155"/>
-      <c r="C28" s="155"/>
-      <c r="D28" s="155"/>
-      <c r="E28" s="155"/>
-      <c r="F28" s="155"/>
-      <c r="G28" s="155"/>
+      <c r="B28" s="129"/>
+      <c r="C28" s="129"/>
+      <c r="D28" s="129"/>
+      <c r="E28" s="129"/>
+      <c r="F28" s="129"/>
+      <c r="G28" s="129"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A29" s="21"/>
-      <c r="B29" s="155"/>
-      <c r="C29" s="155"/>
-      <c r="D29" s="155"/>
-      <c r="E29" s="155"/>
-      <c r="F29" s="155"/>
-      <c r="G29" s="155"/>
+      <c r="B29" s="129"/>
+      <c r="C29" s="129"/>
+      <c r="D29" s="129"/>
+      <c r="E29" s="129"/>
+      <c r="F29" s="129"/>
+      <c r="G29" s="129"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A30" s="21"/>
-      <c r="B30" s="155"/>
-      <c r="C30" s="155"/>
-      <c r="D30" s="155"/>
-      <c r="E30" s="155"/>
-      <c r="F30" s="155"/>
-      <c r="G30" s="155"/>
+      <c r="B30" s="129"/>
+      <c r="C30" s="129"/>
+      <c r="D30" s="129"/>
+      <c r="E30" s="129"/>
+      <c r="F30" s="129"/>
+      <c r="G30" s="129"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A31" s="21"/>
-      <c r="B31" s="155"/>
-      <c r="C31" s="155"/>
-      <c r="D31" s="155"/>
-      <c r="E31" s="155"/>
-      <c r="F31" s="155"/>
-      <c r="G31" s="155"/>
+      <c r="B31" s="129"/>
+      <c r="C31" s="129"/>
+      <c r="D31" s="129"/>
+      <c r="E31" s="129"/>
+      <c r="F31" s="129"/>
+      <c r="G31" s="129"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A32" s="21"/>
-      <c r="B32" s="155"/>
-      <c r="C32" s="155"/>
-      <c r="D32" s="155"/>
-      <c r="E32" s="155"/>
-      <c r="F32" s="155"/>
-      <c r="G32" s="155"/>
+      <c r="B32" s="129"/>
+      <c r="C32" s="129"/>
+      <c r="D32" s="129"/>
+      <c r="E32" s="129"/>
+      <c r="F32" s="129"/>
+      <c r="G32" s="129"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A33" s="21"/>
-      <c r="B33" s="155"/>
-      <c r="C33" s="155"/>
-      <c r="D33" s="155"/>
-      <c r="E33" s="155"/>
-      <c r="F33" s="155"/>
-      <c r="G33" s="155"/>
+      <c r="B33" s="129"/>
+      <c r="C33" s="129"/>
+      <c r="D33" s="129"/>
+      <c r="E33" s="129"/>
+      <c r="F33" s="129"/>
+      <c r="G33" s="129"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A34" s="21"/>
-      <c r="B34" s="155"/>
-      <c r="C34" s="155"/>
-      <c r="D34" s="155"/>
-      <c r="E34" s="155"/>
-      <c r="F34" s="155"/>
-      <c r="G34" s="155"/>
+      <c r="B34" s="129"/>
+      <c r="C34" s="129"/>
+      <c r="D34" s="129"/>
+      <c r="E34" s="129"/>
+      <c r="F34" s="129"/>
+      <c r="G34" s="129"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
-      <c r="B35" s="155"/>
-      <c r="C35" s="155"/>
-      <c r="D35" s="155"/>
-      <c r="E35" s="155"/>
-      <c r="F35" s="155"/>
-      <c r="G35" s="155"/>
+      <c r="B35" s="129"/>
+      <c r="C35" s="129"/>
+      <c r="D35" s="129"/>
+      <c r="E35" s="129"/>
+      <c r="F35" s="129"/>
+      <c r="G35" s="129"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A36" s="21"/>
-      <c r="B36" s="155"/>
-      <c r="C36" s="155"/>
-      <c r="D36" s="155"/>
-      <c r="E36" s="155"/>
-      <c r="F36" s="155"/>
-      <c r="G36" s="155"/>
+      <c r="B36" s="129"/>
+      <c r="C36" s="129"/>
+      <c r="D36" s="129"/>
+      <c r="E36" s="129"/>
+      <c r="F36" s="129"/>
+      <c r="G36" s="129"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A37" s="21"/>
-      <c r="B37" s="155"/>
-      <c r="C37" s="155"/>
-      <c r="D37" s="155"/>
-      <c r="E37" s="155"/>
-      <c r="F37" s="155"/>
-      <c r="G37" s="155"/>
+      <c r="B37" s="129"/>
+      <c r="C37" s="129"/>
+      <c r="D37" s="129"/>
+      <c r="E37" s="129"/>
+      <c r="F37" s="129"/>
+      <c r="G37" s="129"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
-      <c r="B38" s="155"/>
-      <c r="C38" s="155"/>
-      <c r="D38" s="155"/>
-      <c r="E38" s="155"/>
-      <c r="F38" s="155"/>
-      <c r="G38" s="155"/>
+      <c r="B38" s="129"/>
+      <c r="C38" s="129"/>
+      <c r="D38" s="129"/>
+      <c r="E38" s="129"/>
+      <c r="F38" s="129"/>
+      <c r="G38" s="129"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A39" s="21"/>
-      <c r="B39" s="155"/>
-      <c r="C39" s="155"/>
-      <c r="D39" s="155"/>
-      <c r="E39" s="155"/>
-      <c r="F39" s="155"/>
-      <c r="G39" s="155"/>
+      <c r="B39" s="129"/>
+      <c r="C39" s="129"/>
+      <c r="D39" s="129"/>
+      <c r="E39" s="129"/>
+      <c r="F39" s="129"/>
+      <c r="G39" s="129"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A40" s="21"/>
-      <c r="B40" s="155"/>
-      <c r="C40" s="155"/>
-      <c r="D40" s="155"/>
-      <c r="E40" s="155"/>
-      <c r="F40" s="155"/>
-      <c r="G40" s="155"/>
+      <c r="B40" s="129"/>
+      <c r="C40" s="129"/>
+      <c r="D40" s="129"/>
+      <c r="E40" s="129"/>
+      <c r="F40" s="129"/>
+      <c r="G40" s="129"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A41" s="21"/>
-      <c r="B41" s="155"/>
-      <c r="C41" s="155"/>
-      <c r="D41" s="155"/>
-      <c r="E41" s="155"/>
-      <c r="F41" s="155"/>
-      <c r="G41" s="155"/>
+      <c r="B41" s="129"/>
+      <c r="C41" s="129"/>
+      <c r="D41" s="129"/>
+      <c r="E41" s="129"/>
+      <c r="F41" s="129"/>
+      <c r="G41" s="129"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" s="21"/>
-      <c r="B42" s="155"/>
-      <c r="C42" s="155"/>
-      <c r="D42" s="155"/>
-      <c r="E42" s="155"/>
-      <c r="F42" s="155"/>
-      <c r="G42" s="155"/>
+      <c r="B42" s="129"/>
+      <c r="C42" s="129"/>
+      <c r="D42" s="129"/>
+      <c r="E42" s="129"/>
+      <c r="F42" s="129"/>
+      <c r="G42" s="129"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -23045,17 +23595,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="24" x14ac:dyDescent="0.3">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="125" t="s">
         <v>1004</v>
       </c>
       <c r="B1" s="3"/>
-      <c r="C1" s="127" t="s">
+      <c r="C1" s="126" t="s">
         <v>1028</v>
       </c>
-      <c r="D1" s="127" t="s">
+      <c r="D1" s="126" t="s">
         <v>1034</v>
       </c>
-      <c r="E1" s="127" t="s">
+      <c r="E1" s="126" t="s">
         <v>1043</v>
       </c>
       <c r="G1" s="3" t="s">
@@ -23063,7 +23613,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="111" t="s">
+      <c r="A2" s="110" t="s">
         <v>917</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -23081,7 +23631,7 @@
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="3"/>
-      <c r="B3" s="156" t="s">
+      <c r="B3" s="3" t="s">
         <v>1057</v>
       </c>
       <c r="C3" s="16" t="s">
@@ -23095,34 +23645,34 @@
       </c>
     </row>
     <row r="4" spans="1:7" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="159" t="s">
+      <c r="A4" s="132" t="s">
         <v>1059</v>
       </c>
-      <c r="B4" s="159" t="s">
+      <c r="B4" s="132" t="s">
         <v>1002</v>
       </c>
-      <c r="C4" s="159" t="s">
+      <c r="C4" s="132" t="s">
         <v>1002</v>
       </c>
-      <c r="D4" s="159" t="s">
+      <c r="D4" s="132" t="s">
         <v>1002</v>
       </c>
-      <c r="E4" s="159" t="s">
+      <c r="E4" s="132" t="s">
         <v>1002</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="157" t="s">
+      <c r="A5" s="130" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="129"/>
-      <c r="C5" s="158">
+      <c r="B5" s="128"/>
+      <c r="C5" s="131">
         <v>0.74</v>
       </c>
-      <c r="D5" s="158">
+      <c r="D5" s="131">
         <v>0.81</v>
       </c>
-      <c r="E5" s="158">
+      <c r="E5" s="131">
         <v>0.96</v>
       </c>
     </row>
@@ -23130,7 +23680,7 @@
       <c r="A6" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="B6" s="108"/>
+      <c r="B6" s="107"/>
       <c r="C6" s="16"/>
       <c r="D6" s="16"/>
       <c r="E6" s="16"/>
@@ -23139,7 +23689,7 @@
       <c r="A7" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="B7" s="108"/>
+      <c r="B7" s="107"/>
       <c r="C7" s="16"/>
       <c r="D7" s="16"/>
       <c r="E7" s="16"/>
@@ -23148,7 +23698,7 @@
       <c r="A8" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="B8" s="117">
+      <c r="B8" s="116">
         <v>0.9</v>
       </c>
       <c r="C8" s="16"/>
@@ -23159,7 +23709,7 @@
       <c r="A9" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="B9" s="108"/>
+      <c r="B9" s="107"/>
       <c r="C9" s="16"/>
       <c r="D9" s="16"/>
       <c r="E9" s="16"/>
@@ -23168,7 +23718,7 @@
       <c r="A10" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="117">
+      <c r="B10" s="116">
         <v>0</v>
       </c>
       <c r="C10" s="16"/>
@@ -23179,14 +23729,14 @@
       <c r="A11" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="B11" s="108"/>
-      <c r="C11" s="116">
+      <c r="B11" s="107"/>
+      <c r="C11" s="115">
         <v>0.95</v>
       </c>
-      <c r="D11" s="116">
+      <c r="D11" s="115">
         <v>1</v>
       </c>
-      <c r="E11" s="116">
+      <c r="E11" s="115">
         <v>1</v>
       </c>
     </row>
@@ -23194,7 +23744,7 @@
       <c r="A12" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="B12" s="108"/>
+      <c r="B12" s="107"/>
       <c r="C12" s="16"/>
       <c r="D12" s="16"/>
       <c r="E12" s="16"/>
@@ -23203,7 +23753,7 @@
       <c r="A13" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="B13" s="108"/>
+      <c r="B13" s="107"/>
       <c r="C13" s="16"/>
       <c r="D13" s="16"/>
       <c r="E13" s="16"/>
@@ -23212,7 +23762,7 @@
       <c r="A14" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="B14" s="108"/>
+      <c r="B14" s="107"/>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="16"/>
@@ -23221,14 +23771,14 @@
       <c r="A15" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="B15" s="108"/>
-      <c r="C15" s="116">
+      <c r="B15" s="107"/>
+      <c r="C15" s="115">
         <v>0.95</v>
       </c>
-      <c r="D15" s="116">
+      <c r="D15" s="115">
         <v>0.89</v>
       </c>
-      <c r="E15" s="116">
+      <c r="E15" s="115">
         <v>0.89</v>
       </c>
     </row>
@@ -23236,7 +23786,7 @@
       <c r="A16" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="B16" s="108"/>
+      <c r="B16" s="107"/>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
       <c r="E16" s="16"/>
@@ -23245,7 +23795,7 @@
       <c r="A17" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="B17" s="108"/>
+      <c r="B17" s="107"/>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="16"/>
@@ -23254,7 +23804,7 @@
       <c r="A18" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="B18" s="117">
+      <c r="B18" s="116">
         <v>0.9</v>
       </c>
       <c r="C18" s="16"/>
@@ -23265,14 +23815,14 @@
       <c r="A19" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B19" s="108"/>
-      <c r="C19" s="116">
+      <c r="B19" s="107"/>
+      <c r="C19" s="115">
         <v>0</v>
       </c>
-      <c r="D19" s="116">
+      <c r="D19" s="115">
         <v>0.98</v>
       </c>
-      <c r="E19" s="116">
+      <c r="E19" s="115">
         <v>0.98</v>
       </c>
     </row>
@@ -23280,7 +23830,7 @@
       <c r="A20" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B20" s="108"/>
+      <c r="B20" s="107"/>
       <c r="C20" s="16"/>
       <c r="D20" s="16"/>
       <c r="E20" s="16"/>
@@ -23289,7 +23839,7 @@
       <c r="A21" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="B21" s="108"/>
+      <c r="B21" s="107"/>
       <c r="C21" s="16"/>
       <c r="D21" s="16"/>
       <c r="E21" s="16"/>
@@ -23298,7 +23848,7 @@
       <c r="A22" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="B22" s="108"/>
+      <c r="B22" s="107"/>
       <c r="C22" s="16"/>
       <c r="D22" s="16"/>
       <c r="E22" s="16"/>
@@ -23307,7 +23857,7 @@
       <c r="A23" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="B23" s="117">
+      <c r="B23" s="116">
         <v>0.9</v>
       </c>
       <c r="C23" s="16"/>
@@ -23318,7 +23868,7 @@
       <c r="A24" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B24" s="108"/>
+      <c r="B24" s="107"/>
       <c r="C24" s="16"/>
       <c r="D24" s="16"/>
       <c r="E24" s="16"/>
@@ -23327,7 +23877,7 @@
       <c r="A25" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B25" s="117">
+      <c r="B25" s="116">
         <v>0.9</v>
       </c>
       <c r="C25" s="16"/>
@@ -23338,7 +23888,7 @@
       <c r="A26" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="B26" s="108"/>
+      <c r="B26" s="107"/>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
       <c r="E26" s="16"/>
@@ -23347,14 +23897,14 @@
       <c r="A27" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="B27" s="108"/>
-      <c r="C27" s="116">
+      <c r="B27" s="107"/>
+      <c r="C27" s="115">
         <v>0</v>
       </c>
-      <c r="D27" s="116">
+      <c r="D27" s="115">
         <v>0</v>
       </c>
-      <c r="E27" s="116">
+      <c r="E27" s="115">
         <v>0</v>
       </c>
     </row>
@@ -23362,7 +23912,7 @@
       <c r="A28" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="B28" s="108"/>
+      <c r="B28" s="107"/>
       <c r="C28" s="16"/>
       <c r="D28" s="16"/>
       <c r="E28" s="16"/>
@@ -23371,7 +23921,7 @@
       <c r="A29" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="B29" s="108"/>
+      <c r="B29" s="107"/>
       <c r="C29" s="16"/>
       <c r="D29" s="16"/>
       <c r="E29" s="16"/>
@@ -23380,14 +23930,14 @@
       <c r="A30" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B30" s="108"/>
-      <c r="C30" s="116">
+      <c r="B30" s="107"/>
+      <c r="C30" s="115">
         <v>0</v>
       </c>
-      <c r="D30" s="116">
+      <c r="D30" s="115">
         <v>1</v>
       </c>
-      <c r="E30" s="116">
+      <c r="E30" s="115">
         <v>0.96</v>
       </c>
     </row>
@@ -23395,14 +23945,14 @@
       <c r="A31" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B31" s="108"/>
-      <c r="C31" s="116">
+      <c r="B31" s="107"/>
+      <c r="C31" s="115">
         <v>0</v>
       </c>
-      <c r="D31" s="116">
+      <c r="D31" s="115">
         <v>0.32</v>
       </c>
-      <c r="E31" s="116">
+      <c r="E31" s="115">
         <v>0.96</v>
       </c>
     </row>
@@ -23410,7 +23960,7 @@
       <c r="A32" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="B32" s="108"/>
+      <c r="B32" s="107"/>
       <c r="C32" s="16"/>
       <c r="D32" s="16"/>
       <c r="E32" s="16"/>
@@ -23419,7 +23969,7 @@
       <c r="A33" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="B33" s="108"/>
+      <c r="B33" s="107"/>
       <c r="C33" s="16"/>
       <c r="D33" s="16"/>
       <c r="E33" s="16"/>
@@ -23428,7 +23978,7 @@
       <c r="A34" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B34" s="108"/>
+      <c r="B34" s="107"/>
       <c r="C34" s="16"/>
       <c r="D34" s="16"/>
       <c r="E34" s="16"/>
@@ -23437,14 +23987,14 @@
       <c r="A35" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B35" s="108"/>
-      <c r="C35" s="116">
+      <c r="B35" s="107"/>
+      <c r="C35" s="115">
         <v>0</v>
       </c>
-      <c r="D35" s="116">
+      <c r="D35" s="115">
         <v>0</v>
       </c>
-      <c r="E35" s="116">
+      <c r="E35" s="115">
         <v>0</v>
       </c>
     </row>
@@ -23452,7 +24002,7 @@
       <c r="A36" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B36" s="108"/>
+      <c r="B36" s="107"/>
       <c r="C36" s="16"/>
       <c r="D36" s="16"/>
       <c r="E36" s="16"/>
@@ -23461,7 +24011,7 @@
       <c r="A37" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="B37" s="108"/>
+      <c r="B37" s="107"/>
       <c r="C37" s="16"/>
       <c r="D37" s="16"/>
       <c r="E37" s="16"/>
@@ -23470,7 +24020,7 @@
       <c r="A38" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="B38" s="108"/>
+      <c r="B38" s="107"/>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>
       <c r="E38" s="16"/>
@@ -23479,7 +24029,7 @@
       <c r="A39" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="B39" s="117">
+      <c r="B39" s="116">
         <v>0.9</v>
       </c>
       <c r="C39" s="16"/>
@@ -23490,7 +24040,7 @@
       <c r="A40" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="B40" s="108"/>
+      <c r="B40" s="107"/>
       <c r="C40" s="16"/>
       <c r="D40" s="16"/>
       <c r="E40" s="16"/>
@@ -23499,7 +24049,7 @@
       <c r="A41" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B41" s="108"/>
+      <c r="B41" s="107"/>
       <c r="C41" s="16"/>
       <c r="D41" s="16"/>
       <c r="E41" s="16"/>
@@ -23508,7 +24058,7 @@
       <c r="A42" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B42" s="108"/>
+      <c r="B42" s="107"/>
       <c r="C42" s="16"/>
       <c r="D42" s="16"/>
       <c r="E42" s="16"/>
@@ -23517,7 +24067,7 @@
       <c r="A43" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B43" s="108"/>
+      <c r="B43" s="107"/>
       <c r="C43" s="16"/>
       <c r="D43" s="16"/>
       <c r="E43" s="16"/>
@@ -23526,7 +24076,7 @@
       <c r="A44" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B44" s="108"/>
+      <c r="B44" s="107"/>
       <c r="C44" s="16"/>
       <c r="D44" s="16"/>
       <c r="E44" s="16"/>

</xml_diff>